<commit_message>
feat: add live HTTP telemetry simulator; update tracker
scripts/liveSimulator.ts POSTs a reading batch to POST /devices/:id/readings
every 5s (LIVE_SIM_INTERVAL_MS to change it), authenticated with
X-Device-Key like a real device, against the same SIM-DEV-001 device
seedTestData.ts uses. Small per-parameter random drift plus an occasional
simulated value:null/status:"unavailable" reading. Finishes P1-05 — unlike
seedTestData.ts (writes straight into the DB once), this exercises the API
over HTTP on an interval, so SSE consumers (SensorGrid, /telemetry/stream,
/alerts/stream) can be tested against live-arriving data.

Also adds backend/docs/script.md documenting both scripts in one place
(trimming the now-duplicate write-up out of API_REFERENCE.md), and updates
docs/tracker/todo.md + the project tracker to reflect P1-05 as Done.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/docs/tracker/IoT Water Filtration - Project Tracker.xlsx
+++ b/backend/docs/tracker/IoT Water Filtration - Project Tracker.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Project Tracker" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Client Requirements" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Risks &amp; Issues" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Roles" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Dashboard" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Project Tracker" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Client Requirements" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Risks &amp; Issues" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Team Roles" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -430,7 +430,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Phase 2 — Backend API core implemented in TypeScript (auth, telemetry, alerts, test runs, calibration, lab validation, maintenance, settings, devices, users); telemetry ingestion, CSV export, and alert-generation logic remain. Frontend v1 complete; Phase 0 hardware gaps pending.</t>
+          <t>Phase 2 — Backend API core implemented in TypeScript (auth, telemetry, telemetry ingestion, alerts, test runs, calibration, lab validation, maintenance, settings, devices, users). CSV export and automatic alert-generation logic remain. Frontend v1 complete; Phase 0 hardware gaps pending.</t>
         </is>
       </c>
     </row>
@@ -740,7 +740,7 @@
     <row r="28">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>• Backend API implemented (Express + TypeScript, commit 598f0e1) per API ROUTES PLAN — needs team review/approval; telemetry ingestion + CSV export + alert-generation logic still outstanding.</t>
+          <t>• Backend API implemented (Express + TypeScript, commit 46cd55f) per API ROUTES PLAN, including telemetry ingestion — needs team review/approval; CSV export + alert-generation logic still outstanding.</t>
         </is>
       </c>
     </row>
@@ -1426,7 +1426,7 @@
       </c>
       <c r="H13" s="9" t="inlineStr">
         <is>
-          <t>In Progress</t>
+          <t>Done</t>
         </is>
       </c>
       <c r="I13" s="11" t="inlineStr">
@@ -1436,7 +1436,7 @@
       </c>
       <c r="J13" s="9" t="inlineStr">
         <is>
-          <t>Generate fake pre/post pH, turbidity, TDS, temperature, flow and status payloads. backend/scripts/seedTestData.ts generates 5 simulated pre/post reading cycles per test run directly into sensor_readings (pH, turbidity, TDS, temperature, flow rate) for local testing — see docs/API_REFERENCE.md. This seeds the DB directly rather than acting as a live device posting over HTTP; a continuous HTTP-based simulator still depends on the ingestion endpoint in P2-02. Commit 598f0e1 on feature/backend-init.</t>
+          <t>Generate fake pre/post pH, turbidity, TDS, temperature, flow and status payloads. backend/scripts/seedTestData.ts seeds 5 simulated pre/post reading cycles directly into sensor_readings for local testing. backend/scripts/liveSimulator.ts (new) is the continuous version: it POSTs a reading batch to POST /devices/:id/readings every 5s (X-Device-Key auth), with per-parameter drift and occasional simulated unavailable readings, so dashboard live surfaces (SSE, SensorGrid) can be exercised the same way real hardware will drive them. Run via `npm run simulate`. See docs/API_REFERENCE.md.</t>
         </is>
       </c>
       <c r="K13" s="9" t="inlineStr">
@@ -1542,7 +1542,7 @@
       </c>
       <c r="J15" s="9" t="inlineStr">
         <is>
-          <t>Validate device ID, payload types, timestamps and missing fields; save telemetry. Implemented: POST /devices/:id/readings — batched ingestion, validates each reading's category/position/value against the device's registered sensors rows, skips (not fails) invalid/unregistered entries individually, and bumps devices.last_seen_at/connection_state as a heartbeat. Authenticated via a placeholder X-Device-Key shared secret, not the real device-auth decision (PENDING_DECISIONS §8). See docs/API_REFERENCE.md → Devices. Implemented on feature/backend-init (uncommitted as of this tracker update).</t>
+          <t>Validate device ID, payload types, timestamps and missing fields; save telemetry. Implemented: POST /devices/:id/readings — batched ingestion, validates each reading's category/position/value against the device's registered sensors rows, skips (not fails) invalid/unregistered entries individually, and bumps devices.last_seen_at/connection_state as a heartbeat. Authenticated via a placeholder X-Device-Key shared secret, not the real device-auth decision (PENDING_DECISIONS §8). See docs/API_REFERENCE.md → Devices. Committed on feature/backend-init (commit 46cd55f).</t>
         </is>
       </c>
       <c r="K15" s="9" t="inlineStr">

</xml_diff>